<commit_message>
create all activity function
</commit_message>
<xml_diff>
--- a/ZayirAlkhayr/wwwroot/Template/ZAStyle.xlsx
+++ b/ZayirAlkhayr/wwwroot/Template/ZAStyle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\salam\New folder\ZayirAlkhayr\ZayirAlkhayr\ZayirAlkhayr\wwwroot\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D50D3730-9262-4D76-AF3C-EA22C8C1BF08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF0E265-0899-4351-BB2E-4A7E3E648259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t xml:space="preserve">تاريخ التحميل : </t>
+  </si>
+  <si>
+    <t xml:space="preserve">اسم المستخدم : </t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -165,22 +172,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
+      <xdr:colOff>19050</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>9525</xdr:colOff>
+      <xdr:colOff>66675</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>38099</xdr:rowOff>
+      <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09B2F16D-D3FC-45C3-5AA3-C12147B3B38E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{557A49FE-8911-44D7-9C8C-B107CC29ECB9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -202,8 +209,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7534276" y="0"/>
-          <a:ext cx="1285874" cy="666749"/>
+          <a:off x="7553325" y="0"/>
+          <a:ext cx="1323975" cy="666750"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -581,7 +588,9 @@
       <c r="G2" s="4"/>
       <c r="H2" s="6"/>
       <c r="I2" s="1"/>
-      <c r="J2" s="7"/>
+      <c r="J2" s="7" t="s">
+        <v>0</v>
+      </c>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -628,7 +637,9 @@
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="1"/>
-      <c r="J3" s="9"/>
+      <c r="J3" s="9" t="s">
+        <v>1</v>
+      </c>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>

</xml_diff>

<commit_message>
Create Pdf File Service
</commit_message>
<xml_diff>
--- a/ZayirAlkhayr/wwwroot/Template/ZAStyle.xlsx
+++ b/ZayirAlkhayr/wwwroot/Template/ZAStyle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\salam\New folder\ZayirAlkhayr\ZayirAlkhayr\ZayirAlkhayr\wwwroot\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF0E265-0899-4351-BB2E-4A7E3E648259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19C48D70-793B-4E80-BDBF-6B1C61C5FAAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -522,9 +522,10 @@
   <dimension ref="A1:AS2361"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.85546875" style="2" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" style="2" customWidth="1"/>
     <col min="2" max="2" width="17.85546875" style="2" customWidth="1"/>
-    <col min="3" max="7" width="15.85546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="37.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="15.85546875" style="2" customWidth="1"/>
     <col min="8" max="8" width="19.140625" style="2" customWidth="1"/>
     <col min="9" max="9" width="15.85546875" style="2" customWidth="1"/>
     <col min="10" max="10" width="30.5703125" style="2" customWidth="1"/>
@@ -712,20 +713,6 @@
       <c r="AR4" s="1"/>
       <c r="AS4" s="1"/>
     </row>
-    <row r="15" spans="1:45" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:45" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="17" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="29" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="30" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>